<commit_message>
Ajout pour le minou
</commit_message>
<xml_diff>
--- a/APP/02 - DOCUMENTATION/Arbre de puissance.xlsx
+++ b/APP/02 - DOCUMENTATION/Arbre de puissance.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francoisdesautels/Documents/GitHub/S7_APP1/APP/02 - DOCUMENTATION/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DBFC5B3-383D-1A44-A5E2-1A300B876F17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4A1420E-187E-1E49-9B5C-D16C27840403}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="860" windowWidth="41120" windowHeight="25720" xr2:uid="{A5082EB8-EFA9-2544-A712-BC37EFA8A22C}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="55">
   <si>
     <t>24V
 External 
@@ -179,10 +179,31 @@
     <t>ISO USB</t>
   </si>
   <si>
-    <t>R</t>
-  </si>
-  <si>
     <t>CLOCK ETH</t>
+  </si>
+  <si>
+    <t>+24V</t>
+  </si>
+  <si>
+    <t>5V</t>
+  </si>
+  <si>
+    <t>-5V</t>
+  </si>
+  <si>
+    <t>5V_MOT</t>
+  </si>
+  <si>
+    <t>BANK 3</t>
+  </si>
+  <si>
+    <t>Y2 (Clock)</t>
+  </si>
+  <si>
+    <t>U12 (Clock)</t>
+  </si>
+  <si>
+    <t>U5 (Clock)</t>
   </si>
 </sst>
 </file>
@@ -250,7 +271,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -287,6 +308,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="16">
     <border>
@@ -475,7 +502,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -616,6 +643,58 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -639,13 +718,13 @@
     <xdr:from>
       <xdr:col>15</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>63</xdr:row>
+      <xdr:row>109</xdr:row>
       <xdr:rowOff>117230</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>18</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>63</xdr:row>
+      <xdr:row>109</xdr:row>
       <xdr:rowOff>117230</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -692,13 +771,13 @@
     <xdr:from>
       <xdr:col>15</xdr:col>
       <xdr:colOff>5861</xdr:colOff>
-      <xdr:row>69</xdr:row>
+      <xdr:row>115</xdr:row>
       <xdr:rowOff>113323</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>18</xdr:col>
       <xdr:colOff>5861</xdr:colOff>
-      <xdr:row>69</xdr:row>
+      <xdr:row>115</xdr:row>
       <xdr:rowOff>113323</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -745,13 +824,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>60</xdr:row>
+      <xdr:row>106</xdr:row>
       <xdr:rowOff>205154</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>60</xdr:row>
+      <xdr:row>106</xdr:row>
       <xdr:rowOff>205154</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -798,13 +877,13 @@
     <xdr:from>
       <xdr:col>9</xdr:col>
       <xdr:colOff>826477</xdr:colOff>
-      <xdr:row>64</xdr:row>
+      <xdr:row>110</xdr:row>
       <xdr:rowOff>5861</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
       <xdr:colOff>826478</xdr:colOff>
-      <xdr:row>64</xdr:row>
+      <xdr:row>110</xdr:row>
       <xdr:rowOff>5861</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -851,13 +930,13 @@
     <xdr:from>
       <xdr:col>20</xdr:col>
       <xdr:colOff>50801</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>36</xdr:row>
       <xdr:rowOff>160865</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>25</xdr:col>
       <xdr:colOff>8468</xdr:colOff>
-      <xdr:row>25</xdr:row>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>79564</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -901,13 +980,13 @@
     <xdr:from>
       <xdr:col>21</xdr:col>
       <xdr:colOff>301406</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>35</xdr:row>
       <xdr:rowOff>45358</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>23</xdr:col>
       <xdr:colOff>693581</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>36</xdr:row>
       <xdr:rowOff>117442</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1267,37 +1346,51 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA5B481C-62F1-9146-BF47-196E1B7400B6}">
-  <dimension ref="B1:Z77"/>
+  <dimension ref="B1:AH123"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:22" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="7"/>
+      <c r="C2" s="50"/>
+      <c r="F2" s="56" t="s">
+        <v>47</v>
+      </c>
+      <c r="G2" s="25"/>
     </row>
     <row r="3" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="8"/>
-      <c r="C3" s="9"/>
+      <c r="B3" s="51"/>
+      <c r="C3" s="52"/>
+      <c r="F3" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="G3" s="29" t="s">
+        <v>2</v>
+      </c>
       <c r="S3" s="24" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="T3" s="25"/>
       <c r="U3" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="V3" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="10"/>
-      <c r="C4" s="11"/>
-      <c r="S4" s="28" t="s">
+      <c r="B4" s="53"/>
+      <c r="C4" s="54"/>
+      <c r="F4" s="30">
+        <v>24</v>
+      </c>
+      <c r="G4" s="31"/>
+      <c r="S4" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="T4" s="29" t="s">
+      <c r="T4" s="37" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1308,26 +1401,34 @@
       <c r="C5" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="S5" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="T5" s="31"/>
+      <c r="F5" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="G5" s="33"/>
+      <c r="S5" s="38" t="s">
+        <v>25</v>
+      </c>
+      <c r="T5" s="39"/>
     </row>
     <row r="6" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="2"/>
+      <c r="B6" s="2">
+        <v>24</v>
+      </c>
       <c r="C6" s="3"/>
-      <c r="S6" s="32" t="s">
+      <c r="F6" s="34"/>
+      <c r="G6" s="35"/>
+      <c r="S6" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="T6" s="33"/>
+      <c r="T6" s="41"/>
     </row>
     <row r="7" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="15"/>
-      <c r="S7" s="34"/>
-      <c r="T7" s="35"/>
+      <c r="C7" s="27"/>
+      <c r="S7" s="42"/>
+      <c r="T7" s="43"/>
     </row>
     <row r="8" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B8" s="4"/>
@@ -1335,38 +1436,40 @@
     </row>
     <row r="9" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="S9" s="24" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="T9" s="25"/>
     </row>
     <row r="10" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="S10" s="28" t="s">
+      <c r="S10" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="T10" s="29" t="s">
+      <c r="T10" s="37" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="11" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="S11" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="T11" s="31"/>
+      <c r="S11" s="38" t="s">
+        <v>25</v>
+      </c>
+      <c r="T11" s="39"/>
     </row>
     <row r="12" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="S12" s="32" t="s">
+      <c r="S12" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="T12" s="33"/>
+      <c r="T12" s="41"/>
     </row>
     <row r="13" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="S13" s="34"/>
-      <c r="T13" s="35"/>
-    </row>
-    <row r="14" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+      <c r="S13" s="42"/>
+      <c r="T13" s="43"/>
+    </row>
+    <row r="14" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J14" s="55"/>
+    </row>
     <row r="15" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="S15" s="24" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="T15" s="25"/>
       <c r="U15" t="s">
@@ -1377,115 +1480,74 @@
       </c>
     </row>
     <row r="16" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="S16" s="36" t="s">
+      <c r="S16" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="T16" s="37" t="s">
+      <c r="T16" s="29" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="11:26" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="S17" s="38" t="s">
+    <row r="17" spans="19:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="S17" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="T17" s="39"/>
-    </row>
-    <row r="18" spans="11:26" x14ac:dyDescent="0.2">
-      <c r="K18" t="s">
+      <c r="T17" s="31"/>
+    </row>
+    <row r="18" spans="19:22" x14ac:dyDescent="0.2">
+      <c r="S18" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="T18" s="33"/>
+    </row>
+    <row r="19" spans="19:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="S19" s="34"/>
+      <c r="T19" s="35"/>
+    </row>
+    <row r="20" spans="19:22" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="19:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="S21" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="T21" s="25"/>
+    </row>
+    <row r="22" spans="19:22" x14ac:dyDescent="0.2">
+      <c r="S22" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="L18" t="s">
-        <v>46</v>
-      </c>
-      <c r="M18" t="s">
+      <c r="T22" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="N18" t="s">
+    </row>
+    <row r="23" spans="19:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="S23" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="T23" s="31"/>
+    </row>
+    <row r="24" spans="19:22" x14ac:dyDescent="0.2">
+      <c r="S24" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="S18" s="40" t="s">
-        <v>3</v>
-      </c>
-      <c r="T18" s="41"/>
-    </row>
-    <row r="19" spans="11:26" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="K19">
-        <v>3.3</v>
-      </c>
-      <c r="L19">
-        <v>1220</v>
-      </c>
-      <c r="M19">
-        <f>K19/L19</f>
-        <v>2.7049180327868849E-3</v>
-      </c>
-      <c r="N19">
-        <f>M19*K19</f>
-        <v>8.9262295081967199E-3</v>
-      </c>
-      <c r="S19" s="42"/>
-      <c r="T19" s="43"/>
-    </row>
-    <row r="20" spans="11:26" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="11:26" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="S21" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="T21" s="25"/>
-      <c r="U21" t="s">
-        <v>36</v>
-      </c>
-      <c r="V21" t="s">
-        <v>37</v>
-      </c>
-      <c r="W21" t="s">
-        <v>43</v>
-      </c>
-      <c r="X21" t="s">
-        <v>44</v>
-      </c>
-      <c r="Y21" t="s">
-        <v>45</v>
-      </c>
-      <c r="Z21" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="22" spans="11:26" x14ac:dyDescent="0.2">
-      <c r="S22" s="36" t="s">
-        <v>1</v>
-      </c>
-      <c r="T22" s="37" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="23" spans="11:26" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="S23" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="T23" s="39"/>
-    </row>
-    <row r="24" spans="11:26" x14ac:dyDescent="0.2">
-      <c r="S24" s="40" t="s">
-        <v>3</v>
-      </c>
-      <c r="T24" s="41"/>
-    </row>
-    <row r="25" spans="11:26" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="S25" s="42"/>
-      <c r="T25" s="43"/>
-    </row>
-    <row r="26" spans="11:26" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="11:26" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="T24" s="33"/>
+    </row>
+    <row r="25" spans="19:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="S25" s="34"/>
+      <c r="T25" s="35"/>
+    </row>
+    <row r="26" spans="19:22" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="19:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="S27" s="24" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="T27" s="25"/>
       <c r="U27" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="28" spans="11:26" x14ac:dyDescent="0.2">
+      <c r="V27" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="28" spans="19:22" x14ac:dyDescent="0.2">
       <c r="S28" s="36" t="s">
         <v>1</v>
       </c>
@@ -1493,67 +1555,142 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="11:26" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="19:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="S29" s="38" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="T29" s="39"/>
     </row>
-    <row r="30" spans="11:26" x14ac:dyDescent="0.2">
+    <row r="30" spans="19:22" x14ac:dyDescent="0.2">
       <c r="S30" s="40" t="s">
         <v>3</v>
       </c>
       <c r="T30" s="41"/>
     </row>
-    <row r="31" spans="11:26" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="19:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="S31" s="42"/>
       <c r="T31" s="43"/>
     </row>
-    <row r="32" spans="11:26" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="33" spans="19:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="19:22" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="33" spans="11:34" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="S33" s="24" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="T33" s="25"/>
       <c r="U33" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="V33" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="34" spans="19:22" x14ac:dyDescent="0.2">
+        <v>37</v>
+      </c>
+      <c r="W33" t="s">
+        <v>43</v>
+      </c>
+      <c r="X33" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y33" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z33" t="s">
+        <v>46</v>
+      </c>
+      <c r="AA33" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="AB33" s="25"/>
+      <c r="AD33" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE33" s="25"/>
+      <c r="AG33" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="AH33" s="25"/>
+    </row>
+    <row r="34" spans="11:34" x14ac:dyDescent="0.2">
       <c r="S34" s="36" t="s">
         <v>1</v>
       </c>
       <c r="T34" s="37" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="35" spans="19:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="AA34" s="60" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB34" s="61" t="s">
+        <v>2</v>
+      </c>
+      <c r="AD34" s="60" t="s">
+        <v>1</v>
+      </c>
+      <c r="AE34" s="61" t="s">
+        <v>2</v>
+      </c>
+      <c r="AG34" s="60" t="s">
+        <v>1</v>
+      </c>
+      <c r="AH34" s="61" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="11:34" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="S35" s="38" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="T35" s="39"/>
-    </row>
-    <row r="36" spans="19:22" x14ac:dyDescent="0.2">
+      <c r="AA35" s="62" t="s">
+        <v>20</v>
+      </c>
+      <c r="AB35" s="63"/>
+      <c r="AD35" s="62" t="s">
+        <v>20</v>
+      </c>
+      <c r="AE35" s="63"/>
+      <c r="AG35" s="62" t="s">
+        <v>20</v>
+      </c>
+      <c r="AH35" s="63"/>
+    </row>
+    <row r="36" spans="11:34" x14ac:dyDescent="0.2">
       <c r="S36" s="40" t="s">
         <v>3</v>
       </c>
       <c r="T36" s="41"/>
-    </row>
-    <row r="37" spans="19:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="AA36" s="64" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB36" s="65"/>
+      <c r="AD36" s="64" t="s">
+        <v>3</v>
+      </c>
+      <c r="AE36" s="65"/>
+      <c r="AG36" s="64" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH36" s="65"/>
+    </row>
+    <row r="37" spans="11:34" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="S37" s="42"/>
       <c r="T37" s="43"/>
-    </row>
-    <row r="38" spans="19:22" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="19:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="AA37" s="66"/>
+      <c r="AB37" s="67"/>
+      <c r="AD37" s="66"/>
+      <c r="AE37" s="67"/>
+      <c r="AG37" s="66"/>
+      <c r="AH37" s="67"/>
+    </row>
+    <row r="38" spans="11:34" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="11:34" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="S39" s="24" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="T39" s="25"/>
-    </row>
-    <row r="40" spans="19:22" x14ac:dyDescent="0.2">
+      <c r="U39" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="40" spans="11:34" x14ac:dyDescent="0.2">
       <c r="S40" s="36" t="s">
         <v>1</v>
       </c>
@@ -1561,24 +1698,35 @@
         <v>2</v>
       </c>
     </row>
-    <row r="41" spans="19:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="11:34" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="K41" s="57"/>
+      <c r="L41" s="57"/>
       <c r="S41" s="38" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="T41" s="39"/>
     </row>
-    <row r="42" spans="19:22" x14ac:dyDescent="0.2">
+    <row r="42" spans="11:34" x14ac:dyDescent="0.2">
+      <c r="K42" s="58"/>
+      <c r="L42" s="58"/>
       <c r="S42" s="40" t="s">
         <v>3</v>
       </c>
       <c r="T42" s="41"/>
     </row>
-    <row r="43" spans="19:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="11:34" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="K43" s="59"/>
+      <c r="L43" s="59"/>
       <c r="S43" s="42"/>
       <c r="T43" s="43"/>
     </row>
-    <row r="44" spans="19:22" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="19:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="11:34" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="K44" s="58"/>
+      <c r="L44" s="58"/>
+    </row>
+    <row r="45" spans="11:34" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="K45" s="59"/>
+      <c r="L45" s="59"/>
       <c r="S45" s="24" t="s">
         <v>27</v>
       </c>
@@ -1590,7 +1738,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="46" spans="19:22" x14ac:dyDescent="0.2">
+    <row r="46" spans="11:34" x14ac:dyDescent="0.2">
       <c r="S46" s="36" t="s">
         <v>1</v>
       </c>
@@ -1598,33 +1746,33 @@
         <v>2</v>
       </c>
     </row>
-    <row r="47" spans="19:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="11:34" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="S47" s="38" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="T47" s="39"/>
     </row>
-    <row r="48" spans="19:22" x14ac:dyDescent="0.2">
+    <row r="48" spans="11:34" x14ac:dyDescent="0.2">
       <c r="S48" s="40" t="s">
         <v>3</v>
       </c>
       <c r="T48" s="41"/>
     </row>
-    <row r="49" spans="12:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="19:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="S49" s="42"/>
       <c r="T49" s="43"/>
     </row>
-    <row r="50" spans="12:21" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="51" spans="12:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="19:21" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="51" spans="19:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="S51" s="24" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="T51" s="25"/>
       <c r="U51" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="52" spans="12:21" x14ac:dyDescent="0.2">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="52" spans="19:21" x14ac:dyDescent="0.2">
       <c r="S52" s="36" t="s">
         <v>1</v>
       </c>
@@ -1632,37 +1780,30 @@
         <v>2</v>
       </c>
     </row>
-    <row r="53" spans="12:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="19:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="S53" s="38" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="T53" s="39"/>
     </row>
-    <row r="54" spans="12:21" x14ac:dyDescent="0.2">
+    <row r="54" spans="19:21" x14ac:dyDescent="0.2">
       <c r="S54" s="40" t="s">
         <v>3</v>
       </c>
       <c r="T54" s="41"/>
     </row>
-    <row r="55" spans="12:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="19:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="S55" s="42"/>
       <c r="T55" s="43"/>
     </row>
-    <row r="56" spans="12:21" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="12:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="19:21" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="57" spans="19:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="S57" s="24" t="s">
-        <v>29</v>
+        <v>48</v>
       </c>
       <c r="T57" s="25"/>
-      <c r="U57" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="58" spans="12:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="N58" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="O58" s="17"/>
+    </row>
+    <row r="58" spans="19:21" x14ac:dyDescent="0.2">
       <c r="S58" s="36" t="s">
         <v>1</v>
       </c>
@@ -1670,66 +1811,30 @@
         <v>2</v>
       </c>
     </row>
-    <row r="59" spans="12:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="N59" s="19" t="s">
-        <v>4</v>
-      </c>
-      <c r="O59" s="18" t="s">
-        <v>5</v>
-      </c>
+    <row r="59" spans="19:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="S59" s="38" t="s">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="T59" s="39"/>
     </row>
-    <row r="60" spans="12:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="N60" s="20" t="s">
-        <v>7</v>
-      </c>
-      <c r="O60" s="21"/>
+    <row r="60" spans="19:21" x14ac:dyDescent="0.2">
       <c r="S60" s="40" t="s">
         <v>3</v>
       </c>
       <c r="T60" s="41"/>
     </row>
-    <row r="61" spans="12:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="L61" t="s">
-        <v>20</v>
-      </c>
-      <c r="N61" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="O61" s="22" t="s">
-        <v>11</v>
-      </c>
+    <row r="61" spans="19:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="S61" s="42"/>
       <c r="T61" s="43"/>
     </row>
-    <row r="62" spans="12:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="N62" s="2"/>
-      <c r="O62" s="23"/>
-    </row>
-    <row r="63" spans="12:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="N63" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="O63" s="22" t="s">
-        <v>12</v>
-      </c>
-      <c r="S63" s="24" t="s">
-        <v>30</v>
+    <row r="62" spans="19:21" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="63" spans="19:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="S63" s="56" t="s">
+        <v>49</v>
       </c>
       <c r="T63" s="25"/>
-      <c r="U63" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="64" spans="12:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="L64" t="s">
-        <v>24</v>
-      </c>
-      <c r="N64" s="2"/>
-      <c r="O64" s="23"/>
+    </row>
+    <row r="64" spans="19:21" x14ac:dyDescent="0.2">
       <c r="S64" s="36" t="s">
         <v>1</v>
       </c>
@@ -1737,53 +1842,30 @@
         <v>2</v>
       </c>
     </row>
-    <row r="65" spans="14:20" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="N65" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="O65" s="22" t="s">
-        <v>13</v>
-      </c>
+    <row r="65" spans="19:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="S65" s="38" t="s">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="T65" s="39"/>
     </row>
-    <row r="66" spans="14:20" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="N66" s="2"/>
-      <c r="O66" s="23"/>
+    <row r="66" spans="19:21" x14ac:dyDescent="0.2">
       <c r="S66" s="40" t="s">
         <v>3</v>
       </c>
       <c r="T66" s="41"/>
     </row>
-    <row r="67" spans="14:20" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="N67" s="44" t="s">
-        <v>14</v>
-      </c>
-      <c r="O67" s="45"/>
+    <row r="67" spans="19:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="S67" s="42"/>
       <c r="T67" s="43"/>
     </row>
-    <row r="68" spans="14:20" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="N68" s="46"/>
-      <c r="O68" s="47"/>
-    </row>
-    <row r="69" spans="14:20" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="N69" s="48"/>
-      <c r="O69" s="49"/>
+    <row r="68" spans="19:21" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="69" spans="19:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="S69" s="24" t="s">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="T69" s="25"/>
     </row>
-    <row r="70" spans="14:20" x14ac:dyDescent="0.2">
-      <c r="N70" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="O70" s="22" t="s">
-        <v>11</v>
-      </c>
+    <row r="70" spans="19:21" x14ac:dyDescent="0.2">
       <c r="S70" s="36" t="s">
         <v>1</v>
       </c>
@@ -1791,101 +1873,293 @@
         <v>2</v>
       </c>
     </row>
-    <row r="71" spans="14:20" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="N71" s="2"/>
-      <c r="O71" s="23"/>
+    <row r="71" spans="19:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="S71" s="38" t="s">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="T71" s="39"/>
     </row>
-    <row r="72" spans="14:20" x14ac:dyDescent="0.2">
-      <c r="N72" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="O72" s="22" t="s">
-        <v>12</v>
-      </c>
+    <row r="72" spans="19:21" x14ac:dyDescent="0.2">
       <c r="S72" s="40" t="s">
         <v>3</v>
       </c>
       <c r="T72" s="41"/>
     </row>
-    <row r="73" spans="14:20" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="N73" s="2"/>
-      <c r="O73" s="23"/>
+    <row r="73" spans="19:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="S73" s="42"/>
       <c r="T73" s="43"/>
     </row>
-    <row r="74" spans="14:20" x14ac:dyDescent="0.2">
-      <c r="N74" s="12" t="s">
+    <row r="74" spans="19:21" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="75" spans="19:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="S75" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="T75" s="25"/>
+      <c r="U75" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="76" spans="19:21" x14ac:dyDescent="0.2">
+      <c r="S76" s="36" t="s">
+        <v>1</v>
+      </c>
+      <c r="T76" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="77" spans="19:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="S77" s="38" t="s">
+        <v>48</v>
+      </c>
+      <c r="T77" s="39"/>
+    </row>
+    <row r="78" spans="19:21" x14ac:dyDescent="0.2">
+      <c r="S78" s="40" t="s">
+        <v>3</v>
+      </c>
+      <c r="T78" s="41"/>
+    </row>
+    <row r="79" spans="19:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="S79" s="42"/>
+      <c r="T79" s="43"/>
+    </row>
+    <row r="103" spans="12:21" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="104" spans="12:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="N104" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="O104" s="17"/>
+    </row>
+    <row r="105" spans="12:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="N105" s="19" t="s">
+        <v>4</v>
+      </c>
+      <c r="O105" s="18" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="106" spans="12:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="N106" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="O106" s="21"/>
+    </row>
+    <row r="107" spans="12:21" x14ac:dyDescent="0.2">
+      <c r="L107" t="s">
+        <v>20</v>
+      </c>
+      <c r="N107" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="O107" s="22" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="108" spans="12:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="N108" s="2"/>
+      <c r="O108" s="23"/>
+    </row>
+    <row r="109" spans="12:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="N109" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="O109" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="S109" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="T109" s="25"/>
+      <c r="U109" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="110" spans="12:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="L110" t="s">
+        <v>24</v>
+      </c>
+      <c r="N110" s="2"/>
+      <c r="O110" s="23"/>
+      <c r="S110" s="36" t="s">
+        <v>1</v>
+      </c>
+      <c r="T110" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="111" spans="12:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="N111" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="O74" s="22" t="s">
+      <c r="O111" s="22" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="75" spans="14:20" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="N75" s="2"/>
-      <c r="O75" s="23"/>
-    </row>
-    <row r="76" spans="14:20" x14ac:dyDescent="0.2">
-      <c r="N76" s="44" t="s">
+      <c r="S111" s="38" t="s">
+        <v>31</v>
+      </c>
+      <c r="T111" s="39"/>
+    </row>
+    <row r="112" spans="12:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="N112" s="2"/>
+      <c r="O112" s="23"/>
+      <c r="S112" s="40" t="s">
+        <v>3</v>
+      </c>
+      <c r="T112" s="41"/>
+    </row>
+    <row r="113" spans="14:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="N113" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="O76" s="45"/>
-    </row>
-    <row r="77" spans="14:20" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="N77" s="46"/>
-      <c r="O77" s="47"/>
+      <c r="O113" s="45"/>
+      <c r="S113" s="42"/>
+      <c r="T113" s="43"/>
+    </row>
+    <row r="114" spans="14:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="N114" s="46"/>
+      <c r="O114" s="47"/>
+    </row>
+    <row r="115" spans="14:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="N115" s="48"/>
+      <c r="O115" s="49"/>
+      <c r="S115" s="24" t="s">
+        <v>32</v>
+      </c>
+      <c r="T115" s="25"/>
+      <c r="U115" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="116" spans="14:21" x14ac:dyDescent="0.2">
+      <c r="N116" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="O116" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="S116" s="36" t="s">
+        <v>1</v>
+      </c>
+      <c r="T116" s="37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="117" spans="14:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="N117" s="2"/>
+      <c r="O117" s="23"/>
+      <c r="S117" s="38" t="s">
+        <v>31</v>
+      </c>
+      <c r="T117" s="39"/>
+    </row>
+    <row r="118" spans="14:21" x14ac:dyDescent="0.2">
+      <c r="N118" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="O118" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="S118" s="40" t="s">
+        <v>3</v>
+      </c>
+      <c r="T118" s="41"/>
+    </row>
+    <row r="119" spans="14:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="N119" s="2"/>
+      <c r="O119" s="23"/>
+      <c r="S119" s="42"/>
+      <c r="T119" s="43"/>
+    </row>
+    <row r="120" spans="14:21" x14ac:dyDescent="0.2">
+      <c r="N120" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="O120" s="22" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="121" spans="14:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="N121" s="2"/>
+      <c r="O121" s="23"/>
+    </row>
+    <row r="122" spans="14:21" x14ac:dyDescent="0.2">
+      <c r="N122" s="44" t="s">
+        <v>14</v>
+      </c>
+      <c r="O122" s="45"/>
+    </row>
+    <row r="123" spans="14:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="N123" s="46"/>
+      <c r="O123" s="47"/>
     </row>
   </sheetData>
-  <mergeCells count="45">
-    <mergeCell ref="S69:T69"/>
+  <mergeCells count="66">
+    <mergeCell ref="AD33:AE33"/>
+    <mergeCell ref="AD36:AE36"/>
+    <mergeCell ref="AD37:AE37"/>
+    <mergeCell ref="AG33:AH33"/>
+    <mergeCell ref="AG36:AH36"/>
+    <mergeCell ref="AG37:AH37"/>
     <mergeCell ref="S72:T72"/>
     <mergeCell ref="S73:T73"/>
-    <mergeCell ref="N76:O76"/>
-    <mergeCell ref="N77:O77"/>
+    <mergeCell ref="S75:T75"/>
+    <mergeCell ref="S78:T78"/>
+    <mergeCell ref="S79:T79"/>
+    <mergeCell ref="AA33:AB33"/>
+    <mergeCell ref="AA36:AB36"/>
+    <mergeCell ref="AA37:AB37"/>
+    <mergeCell ref="S113:T113"/>
+    <mergeCell ref="S112:T112"/>
+    <mergeCell ref="S109:T109"/>
     <mergeCell ref="S57:T57"/>
     <mergeCell ref="S60:T60"/>
     <mergeCell ref="S61:T61"/>
     <mergeCell ref="S63:T63"/>
     <mergeCell ref="S66:T66"/>
     <mergeCell ref="S67:T67"/>
+    <mergeCell ref="S69:T69"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="S115:T115"/>
+    <mergeCell ref="S118:T118"/>
+    <mergeCell ref="S119:T119"/>
+    <mergeCell ref="N122:O122"/>
+    <mergeCell ref="N123:O123"/>
+    <mergeCell ref="S51:T51"/>
+    <mergeCell ref="S54:T54"/>
+    <mergeCell ref="S55:T55"/>
     <mergeCell ref="S45:T45"/>
     <mergeCell ref="S48:T48"/>
     <mergeCell ref="S49:T49"/>
-    <mergeCell ref="S51:T51"/>
-    <mergeCell ref="S54:T54"/>
-    <mergeCell ref="S55:T55"/>
+    <mergeCell ref="S3:T3"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="S9:T9"/>
+    <mergeCell ref="S12:T12"/>
+    <mergeCell ref="S13:T13"/>
     <mergeCell ref="S33:T33"/>
     <mergeCell ref="S36:T36"/>
     <mergeCell ref="S37:T37"/>
     <mergeCell ref="S39:T39"/>
     <mergeCell ref="S42:T42"/>
     <mergeCell ref="S43:T43"/>
-    <mergeCell ref="S21:T21"/>
-    <mergeCell ref="S24:T24"/>
-    <mergeCell ref="S25:T25"/>
     <mergeCell ref="S27:T27"/>
     <mergeCell ref="S30:T30"/>
     <mergeCell ref="S31:T31"/>
     <mergeCell ref="S15:T15"/>
     <mergeCell ref="S18:T18"/>
     <mergeCell ref="S19:T19"/>
-    <mergeCell ref="S3:T3"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="S7:T7"/>
-    <mergeCell ref="S9:T9"/>
-    <mergeCell ref="S12:T12"/>
-    <mergeCell ref="S13:T13"/>
-    <mergeCell ref="N67:O67"/>
-    <mergeCell ref="N68:O68"/>
+    <mergeCell ref="S21:T21"/>
+    <mergeCell ref="S24:T24"/>
+    <mergeCell ref="S25:T25"/>
+    <mergeCell ref="N113:O113"/>
+    <mergeCell ref="N114:O114"/>
     <mergeCell ref="B2:C4"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B8:C8"/>
-    <mergeCell ref="N58:O58"/>
-    <mergeCell ref="N60:O60"/>
+    <mergeCell ref="N104:O104"/>
+    <mergeCell ref="N106:O106"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>